<commit_message>
Add worked numerical examples to Connected Mode CALC boxes
Chapter 4 now walks A1–A5 / B1 / B2, TimeToTrig, offset clamp, and A4-vs-A2 ping-pong with one teaching set of dBm values. Later feature sheets reuse the same style. Numbers are for understanding only, not a live design.

Co-authored-by: Mohammad Selim <miles4482@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/4G_LTE_Mobility_Management/Connected_Mode_eRAN21.1_Feature_Sheets.xlsx
+++ b/docs/4G_LTE_Mobility_Management/Connected_Mode_eRAN21.1_Feature_Sheets.xlsx
@@ -788,10 +788,10 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="34" customHeight="1">
+    <row r="13" ht="48" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">    •  Command-example dBm in the book (for example A1/A2 −85/−87 dBm, A4 −103 dBm) are not design values. They are not copied into Value.</t>
+          <t xml:space="preserve">    •  Command-example dBm in the book (for example A1/A2 −85/−87 dBm, A4 −103 dBm) are not design values. They are not copied into Value. Chapter 4 has a worked example with numbers for A1–A5 / B1 / offset clamp — those numbers are for understanding only.</t>
         </is>
       </c>
     </row>
@@ -1366,7 +1366,7 @@
       <c r="H15" s="14" t="n"/>
       <c r="I15" s="14" t="n"/>
     </row>
-    <row r="16" ht="110" customHeight="1">
+    <row r="16" ht="112" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
           <t>CELLALGOSWITCH FreqPriorityHoSwitch FreqPriorIFHOSwitch = ON.
@@ -1390,7 +1390,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="28" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Calculation</t>
+          <t xml:space="preserve">  Calculation + example (not a design)</t>
         </is>
       </c>
       <c r="B18" s="29" t="n"/>
@@ -1402,14 +1402,13 @@
       <c r="H18" s="29" t="n"/>
       <c r="I18" s="29" t="n"/>
     </row>
-    <row r="19" ht="110" customHeight="1">
+    <row r="19" ht="80" customHeight="1">
       <c r="A19" s="30" t="inlineStr">
         <is>
-          <t>FreqPri A1: FreqPriInterFreqHoA1ThdRsrp / Rsrq. Trigger quantity FreqPriInterFreqHoA1TrigQuan = RSRP recommended.
-FreqPri A2 (if A2-based mode): FreqPriInterFreqHoA2ThdRsrp / Rsrq.
-Target A4: InterFreqLoadBasedHoA4ThdRsrp (+ FreqPriHoA4ThldRsrpOffset per EARFCN in later versions).
-Waiting: INTRARATHOCOMM FreqPriIFHoWaitingTimer.
-After incoming unnecessary HO: FreqPriInHoProtectionTimer &gt; 0 so the UE is not bounced back at once.</t>
+          <t>FreqPri A1: FreqPriInterFreqHoA1ThdRsrp. Example −90 dBm, Hys 2, Ms −85.  −85 − 2 = −87 &gt; −90 → serving is good, FreqPri may start (same-coverage).
+Target A4: InterFreqLoadBasedHoA4ThdRsrp + FreqPriHoA4ThldRsrpOffset. Example base −105 dBm, per-EARFCN offset +2 dB → used A4 = −103 dBm.
+Mn = −90, Hys = 2.  −92 &gt; −103 → ENTER to high band. Need not beat serving; serving can still be −85 dBm.
+Waiting: FreqPriIFHoWaitingTimer. Example 1 s. After incoming unnecessary HO: FreqPriInHoProtectionTimer example 5 s so the UE is not bounced back at once.</t>
         </is>
       </c>
       <c r="B19" s="29" t="n"/>
@@ -1437,7 +1436,7 @@
       <c r="H21" s="32" t="n"/>
       <c r="I21" s="32" t="n"/>
     </row>
-    <row r="22" ht="110" customHeight="1">
+    <row r="22" ht="96" customHeight="1">
       <c r="A22" s="33" t="inlineStr">
         <is>
           <t>HO_USE_VOIP_FREQ_ALLOWED deselected for all QCIs on the UE when VoipMeasFreqPriSwitch is ON — voice can stop FreqPri meas.
@@ -2442,7 +2441,7 @@
       <c r="H15" s="14" t="n"/>
       <c r="I15" s="14" t="n"/>
     </row>
-    <row r="16" ht="98" customHeight="1">
+    <row r="16" ht="80" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
           <t>Ch.5.3 InterFreqCoverHoSwitch = ON first.
@@ -2464,7 +2463,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="28" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Calculation</t>
+          <t xml:space="preserve">  Calculation + example (not a design)</t>
         </is>
       </c>
       <c r="B18" s="29" t="n"/>
@@ -2476,11 +2475,14 @@
       <c r="H18" s="29" t="n"/>
       <c r="I18" s="29" t="n"/>
     </row>
-    <row r="19" ht="98" customHeight="1">
+    <row r="19" ht="112" customHeight="1">
       <c r="A19" s="30" t="inlineStr">
         <is>
-          <t>Mobility state from HO count in a window (normal / medium / high) as in 3GPP + Huawei speed parameters.
-High-speed: prefer lower-frequency / larger-coverage target. Target still must pass coverage A3 or A4/A5.
+          <t>Mobility state from HO count in a window (normal / medium / high). Confirm the exact parameter names and window in MAE / eRAN21.1 §12.1.2.
+Example: HoNumThd = 4, HighSpeedHoNumThd = 8, SpeedStateJudgePeriod = 60 s, SpeedStateTimer = 120 s, SpeedStateValidTime = 30 s.
+If the eNodeB counts 6 intra-frequency HOs inside the 60 s judge period: 6 ≥ 4 → enter high-speed, start the 120 s timer, and after 30 s apply the high-speed parameter set.
+If the count later stays ≥ 8, keep high-speed. If it falls below 4, return to normal speed.
+High-speed: prefer lower-frequency / larger-coverage target. Target still must pass coverage A3 or A4/A5 (same numbers as Chapter 5).
 Do not set coverage A2 so low that a high-speed UE never leaves a dying small cell — speed HO is not a substitute for A2.</t>
         </is>
       </c>
@@ -2596,7 +2598,7 @@
       <c r="H26" s="32" t="n"/>
       <c r="I26" s="32" t="n"/>
     </row>
-    <row r="27" ht="42" customHeight="1">
+    <row r="27" ht="36" customHeight="1">
       <c r="A27" s="33" t="inlineStr">
         <is>
           <t>FDD. Coverage IFHO already on. Do not confuse with HighSpeedUserRedirectSwitch (railway dedicated network), which is a different option.</t>
@@ -3069,7 +3071,7 @@
       <c r="H20" s="14" t="n"/>
       <c r="I20" s="14" t="n"/>
     </row>
-    <row r="21" ht="56" customHeight="1">
+    <row r="21" ht="36" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
           <t>ENODEBALGOSWITCH MultiOpCtrlSwitch UtranSepOpMobilitySwitch = ON. ADD UTRANNETWORKCAPCFG with MCC, MNC, RncId and the capability bits. Prerequisite: Ch.5.4 UtranPsHoSwitch or UtranRedirectSwitch as required by the policy you want.</t>
@@ -3172,7 +3174,7 @@
       <c r="H27" s="32" t="n"/>
       <c r="I27" s="32" t="n"/>
     </row>
-    <row r="28" ht="42" customHeight="1">
+    <row r="28" ht="36" customHeight="1">
       <c r="A28" s="33" t="inlineStr">
         <is>
           <t>FDD. UTRAN neighbours exist. Flash/ultra-flash/SRVCC licenses if those bits are set. Related: Ch.5.4 and CS Fallback / SRVCC documents.</t>
@@ -3786,7 +3788,7 @@
       <c r="H15" s="14" t="n"/>
       <c r="I15" s="14" t="n"/>
     </row>
-    <row r="16" ht="56" customHeight="1">
+    <row r="16" ht="36" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
           <t>MultiOpCtrlSwitch GeranSepOpMobilitySwitch = ON (confirm exact bit in MAE). Configure per-BSC GERAN capabilities. Prerequisite: Ch.5.5 GeranRedirectSwitch (and related GERAN HO switches) already match the policy you want.</t>
@@ -3889,7 +3891,7 @@
       <c r="H22" s="32" t="n"/>
       <c r="I22" s="32" t="n"/>
     </row>
-    <row r="23" ht="42" customHeight="1">
+    <row r="23" ht="36" customHeight="1">
       <c r="A23" s="33" t="inlineStr">
         <is>
           <t>GERAN NRT present. Related CS Fallback document for SI-by-RIM / CCO. TDD ID is TDLOFD-131210.</t>
@@ -4321,7 +4323,7 @@
       <c r="H15" s="14" t="n"/>
       <c r="I15" s="14" t="n"/>
     </row>
-    <row r="16" ht="42" customHeight="1">
+    <row r="16" ht="36" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
           <t>There is no switch in Chapter 3. Configure Chapter 4 first, then the feature chapter you need.</t>
@@ -4585,7 +4587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I82"/>
+  <dimension ref="A1:I91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4750,7 +4752,7 @@
       <c r="H23" s="14" t="n"/>
       <c r="I23" s="14" t="n"/>
     </row>
-    <row r="24" ht="110" customHeight="1">
+    <row r="24" ht="80" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
           <t>Neighbour frequency: FREQ_MEAS_FLAG selected. HO_TRG_FREQ_FORBID_MEAS_FLAG deselected for required HO targets.
@@ -4873,7 +4875,7 @@
       <c r="H37" s="29" t="n"/>
       <c r="I37" s="29" t="n"/>
     </row>
-    <row r="38" ht="110" customHeight="1">
+    <row r="38" ht="160" customHeight="1">
       <c r="A38" s="30" t="inlineStr">
         <is>
           <t>A1  Ms − Hys &gt; Thresh     serving becomes good (stops coverage measurement; can start FreqPri)
@@ -4884,7 +4886,7 @@
 B1  Mn + Ofn − Hys &gt; Thresh     IRAT neighbour absolutely good
 B2  Ms + Hys &lt; Th1  AND  Mn + Ofn − Hys &gt; Th2     IRAT coverage pair
 Ofn / Ofs = frequency offset. Ocn / Ocs = CellIndividualOffset (CIO). Off = A3 offset. Hys = hysteresis of that event.
-QCI/operator/SPID offsets are added to the base threshold, then clamped. Example: A3InterFreqHoA2ThdRsrp + SPID factor, then MAX(−140, MIN(−43, result)).</t>
+QCI/operator/SPID offsets are added to the base threshold, then clamped: MAX(−140, MIN(−43, result)) for RSRP.</t>
         </is>
       </c>
       <c r="B38" s="29" t="n"/>
@@ -4896,739 +4898,447 @@
       <c r="H38" s="29" t="n"/>
       <c r="I38" s="29" t="n"/>
     </row>
-    <row r="39" ht="58" customHeight="1">
-      <c r="A39" s="8" t="inlineStr">
+    <row r="39" ht="6" customHeight="1"/>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Example with values  ·  for understanding only  ·  not a live design  ·  not the book MML −85/−87/−103 dBm</t>
+        </is>
+      </c>
+      <c r="B40" s="29" t="n"/>
+      <c r="C40" s="29" t="n"/>
+      <c r="D40" s="29" t="n"/>
+      <c r="E40" s="29" t="n"/>
+      <c r="F40" s="29" t="n"/>
+      <c r="G40" s="29" t="n"/>
+      <c r="H40" s="29" t="n"/>
+      <c r="I40" s="29" t="n"/>
+    </row>
+    <row r="41" ht="128" customHeight="1">
+      <c r="A41" s="30" t="inlineStr">
+        <is>
+          <t>One teaching set so the arithmetic is visible. Calibrate real cells from MR. Later chapters re-use the same idea.
+Assume: Ms = −95 dBm (serving RSRP), Mn = −90 dBm (neighbour RSRP), Hys = 2 dB, Ofn = Ofs = 0, Ocn = Ocs = 0, Off = 2 dB, TimeToTrig = 320 ms.
+A1  Thresh = −100 dBm.   Ms − Hys = −95 − 2 = −97.   −97 &gt; −100 → ENTER. Serving is good. Coverage measurement can stop.
+     If Ms = −105 dBm: −105 − 2 = −107.   −107 &gt; −100 → NO. A1 does not enter.
+A2  Thresh = −100 dBm.   Ms + Hys = −95 + 2 = −93.   −93 &lt; −100 → NO. Serving is not poor. Inter-frequency measurement does not start.
+     If Ms = −105 dBm: −105 + 2 = −103.   −103 &lt; −100 → ENTER. Start inter-frequency / IRAT measurement.
+TimeToTrig. The entering condition must stay true for 320 ms. If it is true for 200 ms and then Ms recovers, the timer resets and no report is sent.</t>
+        </is>
+      </c>
+      <c r="B41" s="29" t="n"/>
+      <c r="C41" s="29" t="n"/>
+      <c r="D41" s="29" t="n"/>
+      <c r="E41" s="29" t="n"/>
+      <c r="F41" s="29" t="n"/>
+      <c r="G41" s="29" t="n"/>
+      <c r="H41" s="29" t="n"/>
+      <c r="I41" s="29" t="n"/>
+    </row>
+    <row r="42" ht="6" customHeight="1"/>
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Same teaching set  ·  A3 / A4 / A5  ·  still not a design</t>
+        </is>
+      </c>
+      <c r="B43" s="29" t="n"/>
+      <c r="C43" s="29" t="n"/>
+      <c r="D43" s="29" t="n"/>
+      <c r="E43" s="29" t="n"/>
+      <c r="F43" s="29" t="n"/>
+      <c r="G43" s="29" t="n"/>
+      <c r="H43" s="29" t="n"/>
+      <c r="I43" s="29" t="n"/>
+    </row>
+    <row r="44" ht="128" customHeight="1">
+      <c r="A44" s="30" t="inlineStr">
+        <is>
+          <t>A3  Left = Mn + Ofn + Ocn − Hys = −90 − 2 = −92.   Right = Ms + Ofs + Ocs + Off = −95 + 2 = −93.   −92 &gt; −93 → ENTER. Neighbour is relatively better.
+     If Off = 6 dB: Right = −89.   −92 &gt; −89 → NO. Larger A3 offset makes intra-frequency HO harder.
+     If CIO Ocn = +3 dB: Left = −90 + 3 − 2 = −89.   −89 &gt; −93 → still ENTER, and the neighbour looks 3 dB better.
+A4  Thresh = −105 dBm.   Mn + Ofn + Ocn − Hys = −92.   −92 &gt; −105 → ENTER. Neighbour is absolutely good enough (need not beat serving).
+     If Mn = −110 dBm: −110 − 2 = −112.   −112 &gt; −105 → NO. Target is not good enough.
+A5  Th1 = −110 dBm, Th2 = −105 dBm.   Ms + Hys = −93 &lt; −110? NO. Serving is not poor, so A5 does not enter even though the neighbour is good.
+     If Ms = −115 dBm: −115 + 2 = −113 &lt; −110 YES, and −92 &gt; −105 YES → ENTER. Serving poor AND neighbour good.</t>
+        </is>
+      </c>
+      <c r="B44" s="29" t="n"/>
+      <c r="C44" s="29" t="n"/>
+      <c r="D44" s="29" t="n"/>
+      <c r="E44" s="29" t="n"/>
+      <c r="F44" s="29" t="n"/>
+      <c r="G44" s="29" t="n"/>
+      <c r="H44" s="29" t="n"/>
+      <c r="I44" s="29" t="n"/>
+    </row>
+    <row r="45" ht="6" customHeight="1"/>
+    <row r="46" ht="18" customHeight="1">
+      <c r="A46" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Same teaching set  ·  B1 / B2, offset clamp, A4 vs coverage A2</t>
+        </is>
+      </c>
+      <c r="B46" s="29" t="n"/>
+      <c r="C46" s="29" t="n"/>
+      <c r="D46" s="29" t="n"/>
+      <c r="E46" s="29" t="n"/>
+      <c r="F46" s="29" t="n"/>
+      <c r="G46" s="29" t="n"/>
+      <c r="H46" s="29" t="n"/>
+      <c r="I46" s="29" t="n"/>
+    </row>
+    <row r="47" ht="160" customHeight="1">
+      <c r="A47" s="30" t="inlineStr">
+        <is>
+          <t>B1  IRAT Mn = −92 (configured IRAT quantity), Ofn = 0, Hys = 2, Thresh = −100.   −92 − 2 = −94.   −94 &gt; −100 → ENTER.
+B2  Serving A2-style Th1 = −110, IRAT B1-style Th2 = −100.   Ms = −115: −115 + 2 = −113 &lt; −110 YES, and −94 &gt; −100 YES → ENTER.
+     If Ms = −95: −93 &lt; −110? NO. B2 does not enter even if the IRAT neighbour is good.
+Offset then clamp (A2 RSRP). Base A3InterFreqHoA2ThdRsrp = −100 dBm. SPID factor = +6 dB. Result = −94. MAX(−140, MIN(−43, −94)) = −94 dBm. Used A2 = −94 dBm.
+     If SPID factor = +70 dB: −100 + 70 = −30 → clamp to −43 dBm (cannot go above −43).
+     If SPID factor = −50 dB: −100 − 50 = −150 → clamp to −140 dBm (cannot go below −140).
+A4 vs coverage A2 (ping-pong). ‘A4 better than A2’ means a higher RSRP requirement: A4_thd &gt; A2_thd (for example A4 = −105, A2 = −110).
+     Safe pair: A2 = −110 dBm, A4 = −105 dBm, Mn = −102 dBm. A4: −102 − 2 = −104 &gt; −105 → HO. After HO, serving = −102. A2: −102 + 2 = −100 &lt; −110? NO. Coverage measurement does not start.
+     Unsafe pair: A2 = −100 dBm, A4 = −110 dBm, Mn = −107 dBm. A4: −107 − 2 = −109 &gt; −110 → HO. After HO, serving = −107. A2: −107 + 2 = −105 &lt; −100 YES. Coverage measurement starts at once — ping-pong.</t>
+        </is>
+      </c>
+      <c r="B47" s="29" t="n"/>
+      <c r="C47" s="29" t="n"/>
+      <c r="D47" s="29" t="n"/>
+      <c r="E47" s="29" t="n"/>
+      <c r="F47" s="29" t="n"/>
+      <c r="G47" s="29" t="n"/>
+      <c r="H47" s="29" t="n"/>
+      <c r="I47" s="29" t="n"/>
+    </row>
+    <row r="48" ht="58" customHeight="1">
+      <c r="A48" s="8" t="inlineStr">
         <is>
           <t>A1/A2 Hys and TTT: InterFreqHoGroup.InterFreqHoA1A2Hyst / InterFreqHoA1A2TimeToTrig. A3 Off: IntraFreqHoA3Offset or InterFreqHoA3Offset. A4 Hys/TTT: InterFreqHoA4Hyst / InterFreqHoA4TimeToTrig.</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="10" customHeight="1"/>
-    <row r="41" ht="22" customHeight="1">
-      <c r="A41" s="21" t="inlineStr">
+    <row r="49" ht="10" customHeight="1"/>
+    <row r="50" ht="22" customHeight="1">
+      <c r="A50" s="21" t="inlineStr">
         <is>
           <t>4.1.4  Measurement objects and SMeasure</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="4" customHeight="1"/>
-    <row r="43" ht="58" customHeight="1">
-      <c r="A43" s="8" t="inlineStr">
+    <row r="51" ht="4" customHeight="1"/>
+    <row r="52" ht="58" customHeight="1">
+      <c r="A52" s="8" t="inlineStr">
         <is>
           <t>The eNodeB filters blacklisted cells, NoHoFlag neighbours, and forbidden TA/LA. Frequencies are picked in descending priority. If the highest priority maps to several frequencies, the pick among them is random when over the object cap.</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="6" customHeight="1"/>
-    <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="31" t="inlineStr">
+    <row r="53" ht="6" customHeight="1"/>
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">  Conditions</t>
         </is>
       </c>
-      <c r="B45" s="32" t="n"/>
-      <c r="C45" s="32" t="n"/>
-      <c r="D45" s="32" t="n"/>
-      <c r="E45" s="32" t="n"/>
-      <c r="F45" s="32" t="n"/>
-      <c r="G45" s="32" t="n"/>
-      <c r="H45" s="32" t="n"/>
-      <c r="I45" s="32" t="n"/>
-    </row>
-    <row r="46" ht="98" customHeight="1">
-      <c r="A46" s="33" t="inlineStr">
+      <c r="B54" s="32" t="n"/>
+      <c r="C54" s="32" t="n"/>
+      <c r="D54" s="32" t="n"/>
+      <c r="E54" s="32" t="n"/>
+      <c r="F54" s="32" t="n"/>
+      <c r="G54" s="32" t="n"/>
+      <c r="H54" s="32" t="n"/>
+      <c r="I54" s="32" t="n"/>
+    </row>
+    <row r="55" ht="64" customHeight="1">
+      <c r="A55" s="33" t="inlineStr">
         <is>
           <t>SMeasure (HOMEASCOMM): if serving RSRP is above SMeasure, the UE may skip intra/inter/IRAT measurement. A too-high SMeasure silently kills A4.
 Measurement gap steals DL TTIs. AutoGap / gap pattern must be acceptable for VoLTE and old UEs.
 Algorithm measurement priority: voice/CSFB &gt; necessary coverage &gt; unnecessary single-UE HO &gt; ANR sampling. MEAS_OBJ_PREEMPT_SW allows a higher-priority algorithm to take the gap.</t>
         </is>
       </c>
-      <c r="B46" s="32" t="n"/>
-      <c r="C46" s="32" t="n"/>
-      <c r="D46" s="32" t="n"/>
-      <c r="E46" s="32" t="n"/>
-      <c r="F46" s="32" t="n"/>
-      <c r="G46" s="32" t="n"/>
-      <c r="H46" s="32" t="n"/>
-      <c r="I46" s="32" t="n"/>
-    </row>
-    <row r="47" ht="10" customHeight="1"/>
-    <row r="48" ht="22" customHeight="1">
-      <c r="A48" s="21" t="inlineStr">
+      <c r="B55" s="32" t="n"/>
+      <c r="C55" s="32" t="n"/>
+      <c r="D55" s="32" t="n"/>
+      <c r="E55" s="32" t="n"/>
+      <c r="F55" s="32" t="n"/>
+      <c r="G55" s="32" t="n"/>
+      <c r="H55" s="32" t="n"/>
+      <c r="I55" s="32" t="n"/>
+    </row>
+    <row r="56" ht="10" customHeight="1"/>
+    <row r="57" ht="22" customHeight="1">
+      <c r="A57" s="21" t="inlineStr">
         <is>
           <t>4.1.6–4.1.8  Admit, execute, punish</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="4" customHeight="1"/>
-    <row r="50" ht="44" customHeight="1">
-      <c r="A50" s="8" t="inlineStr">
+    <row r="58" ht="4" customHeight="1"/>
+    <row r="59" ht="44" customHeight="1">
+      <c r="A59" s="8" t="inlineStr">
         <is>
           <t>Necessary: any QCI. Unnecessary offload: all QCIs. Prep fail is often admission or X2, not RF. Penalty timers after fail: do not treat every prep fail as an A4 problem.</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="22" t="inlineStr">
+    <row r="60" ht="18" customHeight="1">
+      <c r="A60" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">  Advantage</t>
         </is>
       </c>
-      <c r="B51" s="23" t="n"/>
-      <c r="C51" s="23" t="n"/>
-      <c r="D51" s="24" t="inlineStr">
+      <c r="B60" s="23" t="n"/>
+      <c r="C60" s="23" t="n"/>
+      <c r="D60" s="24" t="inlineStr">
         <is>
           <t xml:space="preserve">  Limitation</t>
         </is>
       </c>
-      <c r="E51" s="25" t="n"/>
-      <c r="F51" s="25" t="n"/>
-      <c r="G51" s="25" t="n"/>
-      <c r="H51" s="25" t="n"/>
-      <c r="I51" s="25" t="n"/>
-    </row>
-    <row r="52" ht="20" customHeight="1">
-      <c r="A52" s="26" t="inlineStr">
+      <c r="E60" s="25" t="n"/>
+      <c r="F60" s="25" t="n"/>
+      <c r="G60" s="25" t="n"/>
+      <c r="H60" s="25" t="n"/>
+      <c r="I60" s="25" t="n"/>
+    </row>
+    <row r="61" ht="20" customHeight="1">
+      <c r="A61" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">    •  One event set serves every later feature.</t>
         </is>
       </c>
-      <c r="B52" s="23" t="n"/>
-      <c r="C52" s="23" t="n"/>
-      <c r="D52" s="27" t="inlineStr">
+      <c r="B61" s="23" t="n"/>
+      <c r="C61" s="23" t="n"/>
+      <c r="D61" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">    •  Object-cap random drop is not MLB.</t>
         </is>
       </c>
-      <c r="E52" s="25" t="n"/>
-      <c r="F52" s="25" t="n"/>
-      <c r="G52" s="25" t="n"/>
-      <c r="H52" s="25" t="n"/>
-      <c r="I52" s="25" t="n"/>
-    </row>
-    <row r="53" ht="20" customHeight="1">
-      <c r="A53" s="26" t="inlineStr">
+      <c r="E61" s="25" t="n"/>
+      <c r="F61" s="25" t="n"/>
+      <c r="G61" s="25" t="n"/>
+      <c r="H61" s="25" t="n"/>
+      <c r="I61" s="25" t="n"/>
+    </row>
+    <row r="62" ht="20" customHeight="1">
+      <c r="A62" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">    •  QCI-specific Hys/TTT possible.</t>
         </is>
       </c>
-      <c r="B53" s="23" t="n"/>
-      <c r="C53" s="23" t="n"/>
-      <c r="D53" s="27" t="inlineStr">
+      <c r="B62" s="23" t="n"/>
+      <c r="C62" s="23" t="n"/>
+      <c r="D62" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">    •  RSRQ as trigger oscillates with load.</t>
         </is>
       </c>
-      <c r="E53" s="25" t="n"/>
-      <c r="F53" s="25" t="n"/>
-      <c r="G53" s="25" t="n"/>
-      <c r="H53" s="25" t="n"/>
-      <c r="I53" s="25" t="n"/>
-    </row>
-    <row r="54" ht="20" customHeight="1">
-      <c r="A54" s="26" t="inlineStr"/>
-      <c r="B54" s="23" t="n"/>
-      <c r="C54" s="23" t="n"/>
-      <c r="D54" s="27" t="inlineStr">
+      <c r="E62" s="25" t="n"/>
+      <c r="F62" s="25" t="n"/>
+      <c r="G62" s="25" t="n"/>
+      <c r="H62" s="25" t="n"/>
+      <c r="I62" s="25" t="n"/>
+    </row>
+    <row r="63" ht="20" customHeight="1">
+      <c r="A63" s="26" t="inlineStr"/>
+      <c r="B63" s="23" t="n"/>
+      <c r="C63" s="23" t="n"/>
+      <c r="D63" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">    •  Blind mode has higher access-failure risk.</t>
         </is>
       </c>
-      <c r="E54" s="25" t="n"/>
-      <c r="F54" s="25" t="n"/>
-      <c r="G54" s="25" t="n"/>
-      <c r="H54" s="25" t="n"/>
-      <c r="I54" s="25" t="n"/>
-    </row>
-    <row r="55" ht="14" customHeight="1"/>
-    <row r="56" ht="24" customHeight="1">
-      <c r="A56" s="7" t="inlineStr">
+      <c r="E63" s="25" t="n"/>
+      <c r="F63" s="25" t="n"/>
+      <c r="G63" s="25" t="n"/>
+      <c r="H63" s="25" t="n"/>
+      <c r="I63" s="25" t="n"/>
+    </row>
+    <row r="64" ht="14" customHeight="1"/>
+    <row r="65" ht="24" customHeight="1">
+      <c r="A65" s="7" t="inlineStr">
         <is>
           <t>Combined summary</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="6" customHeight="1"/>
-    <row r="58" ht="58" customHeight="1">
-      <c r="A58" s="8" t="inlineStr">
+    <row r="66" ht="6" customHeight="1"/>
+    <row r="67" ht="58" customHeight="1">
+      <c r="A67" s="8" t="inlineStr">
         <is>
           <t>Fix flags, NRT, object cap, SMeasure and A2 family before any dBm. RSRP trigger. A4 better than coverage A2. A4 TTT ≠ 5120 ms if Ch.6 / Ch.9 / Ch.11 inter-frequency A4 is required. Then open the feature sheet.</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="14" customHeight="1"/>
-    <row r="60" ht="24" customHeight="1">
-      <c r="A60" s="7" t="inlineStr">
+    <row r="68" ht="14" customHeight="1"/>
+    <row r="69" ht="24" customHeight="1">
+      <c r="A69" s="7" t="inlineStr">
         <is>
           <t>Parameter list</t>
         </is>
       </c>
     </row>
-    <row r="61" ht="6" customHeight="1"/>
-    <row r="62" ht="22" customHeight="1">
-      <c r="A62" s="16" t="inlineStr">
+    <row r="70" ht="6" customHeight="1"/>
+    <row r="71" ht="22" customHeight="1">
+      <c r="A71" s="16" t="inlineStr">
         <is>
           <t>SN</t>
         </is>
       </c>
-      <c r="B62" s="16" t="inlineStr">
+      <c r="B71" s="16" t="inlineStr">
         <is>
           <t>MO</t>
         </is>
       </c>
-      <c r="C62" s="16" t="inlineStr">
+      <c r="C71" s="16" t="inlineStr">
         <is>
           <t>Parameter</t>
         </is>
       </c>
-      <c r="D62" s="16" t="inlineStr">
+      <c r="D71" s="16" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="E62" s="16" t="inlineStr">
+      <c r="E71" s="16" t="inlineStr">
         <is>
           <t>Comment</t>
         </is>
       </c>
-      <c r="F62" s="16" t="inlineStr">
+      <c r="F71" s="16" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="G62" s="16" t="inlineStr">
+      <c r="G71" s="16" t="inlineStr">
         <is>
           <t>Sub-group</t>
         </is>
       </c>
-      <c r="H62" s="16" t="inlineStr">
+      <c r="H71" s="16" t="inlineStr">
         <is>
           <t>Parameter Meaning</t>
         </is>
       </c>
-      <c r="I62" s="16" t="inlineStr">
+      <c r="I71" s="16" t="inlineStr">
         <is>
           <t>Reference</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="58" customHeight="1">
-      <c r="A63" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="B63" s="18" t="inlineStr">
-        <is>
-          <t>EUTRANINTERNFREQ</t>
-        </is>
-      </c>
-      <c r="C63" s="18" t="inlineStr">
-        <is>
-          <t>FREQ_MEAS_FLAG</t>
-        </is>
-      </c>
-      <c r="D63" s="19" t="inlineStr">
-        <is>
-          <t>selected</t>
-        </is>
-      </c>
-      <c r="E63" s="18" t="inlineStr">
-        <is>
-          <t>Frequency must be measured. Silent no-HO if off.</t>
-        </is>
-      </c>
-      <c r="F63" s="17" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G63" s="18" t="inlineStr">
-        <is>
-          <t>4.1.4</t>
-        </is>
-      </c>
-      <c r="H63" s="18" t="inlineStr">
-        <is>
-          <t>Whether the UE is configured to measure this E-UTRAN frequency in connected mode.</t>
-        </is>
-      </c>
-      <c r="I63" s="18" t="inlineStr">
-        <is>
-          <t>LBFD-002018  ·  Mobility Management in Connected Mode Feature Parameter Description  ·  eRAN21.1 Issue 08  ·  §4.1.4</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" ht="58" customHeight="1">
-      <c r="A64" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="B64" s="18" t="inlineStr">
-        <is>
-          <t>EUTRANINTERNFREQ</t>
-        </is>
-      </c>
-      <c r="C64" s="18" t="inlineStr">
-        <is>
-          <t>HO_TRG_FREQ_FORBID_MEAS_FLAG</t>
-        </is>
-      </c>
-      <c r="D64" s="19" t="inlineStr">
-        <is>
-          <t>deselected</t>
-        </is>
-      </c>
-      <c r="E64" s="18" t="inlineStr">
-        <is>
-          <t>Must be off for required HO targets.</t>
-        </is>
-      </c>
-      <c r="F64" s="17" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G64" s="18" t="inlineStr">
-        <is>
-          <t>4.1.4</t>
-        </is>
-      </c>
-      <c r="H64" s="18" t="inlineStr">
-        <is>
-          <t>If selected, this frequency is forbidden as a handover target even if measured.</t>
-        </is>
-      </c>
-      <c r="I64" s="18" t="inlineStr">
-        <is>
-          <t>LBFD-002018  ·  Mobility Management in Connected Mode Feature Parameter Description  ·  eRAN21.1 Issue 08  ·  §4.1.4</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="58" customHeight="1">
-      <c r="A65" s="17" t="n">
-        <v>3</v>
-      </c>
-      <c r="B65" s="18" t="inlineStr">
-        <is>
-          <t>EUTRANINTERFREQNCELL</t>
-        </is>
-      </c>
-      <c r="C65" s="18" t="inlineStr">
-        <is>
-          <t>NoHoFlag</t>
-        </is>
-      </c>
-      <c r="D65" s="19" t="inlineStr">
-        <is>
-          <t>PERMIT_HO</t>
-        </is>
-      </c>
-      <c r="E65" s="18" t="inlineStr">
-        <is>
-          <t>Neighbour allowed as HO target.</t>
-        </is>
-      </c>
-      <c r="F65" s="17" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G65" s="18" t="inlineStr">
-        <is>
-          <t>4.1.4</t>
-        </is>
-      </c>
-      <c r="H65" s="18" t="inlineStr">
-        <is>
-          <t>Per-neighbour flag allowing or prohibiting handover to that cell.</t>
-        </is>
-      </c>
-      <c r="I65" s="18" t="inlineStr">
-        <is>
-          <t>LBFD-002018  ·  Mobility Management in Connected Mode Feature Parameter Description  ·  eRAN21.1 Issue 08  ·  §4.1.4</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="58" customHeight="1">
-      <c r="A66" s="17" t="n">
-        <v>4</v>
-      </c>
-      <c r="B66" s="18" t="inlineStr">
-        <is>
-          <t>CELLUEMEASCONTROLCFG</t>
-        </is>
-      </c>
-      <c r="C66" s="18" t="inlineStr">
-        <is>
-          <t>MaxNonIntraMeasObjNum</t>
-        </is>
-      </c>
-      <c r="D66" s="19" t="inlineStr">
-        <is>
-          <t>≥ needed objects</t>
-        </is>
-      </c>
-      <c r="E66" s="18" t="inlineStr">
-        <is>
-          <t>Over cap: equal-priority objects drop at random.</t>
-        </is>
-      </c>
-      <c r="F66" s="17" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G66" s="18" t="inlineStr">
-        <is>
-          <t>4.1.4</t>
-        </is>
-      </c>
-      <c r="H66" s="18" t="inlineStr">
-        <is>
-          <t>Maximum number of non-intra-frequency measurement objects the eNodeB may deliver to a UE.</t>
-        </is>
-      </c>
-      <c r="I66" s="18" t="inlineStr">
-        <is>
-          <t>LBFD-002018  ·  Mobility Management in Connected Mode Feature Parameter Description  ·  eRAN21.1 Issue 08  ·  Table 4-3</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="58" customHeight="1">
-      <c r="A67" s="17" t="n">
-        <v>5</v>
-      </c>
-      <c r="B67" s="18" t="inlineStr">
-        <is>
-          <t>CELLUEMEASCONTROLCFG</t>
-        </is>
-      </c>
-      <c r="C67" s="18" t="inlineStr">
-        <is>
-          <t>MaxEutranFddMeasFreqNum</t>
-        </is>
-      </c>
-      <c r="D67" s="19" t="inlineStr">
-        <is>
-          <t>≥ needed FDD freqs</t>
-        </is>
-      </c>
-      <c r="E67" s="18" t="inlineStr">
-        <is>
-          <t>Same random-drop risk for FDD.</t>
-        </is>
-      </c>
-      <c r="F67" s="17" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G67" s="18" t="inlineStr">
-        <is>
-          <t>4.1.4</t>
-        </is>
-      </c>
-      <c r="H67" s="18" t="inlineStr">
-        <is>
-          <t>Maximum number of neighbouring E-UTRAN FDD frequencies that can be delivered for measurement.</t>
-        </is>
-      </c>
-      <c r="I67" s="18" t="inlineStr">
-        <is>
-          <t>LBFD-002018  ·  Mobility Management in Connected Mode Feature Parameter Description  ·  eRAN21.1 Issue 08  ·  Table 4-3</t>
-        </is>
-      </c>
-    </row>
-    <row r="68" ht="58" customHeight="1">
-      <c r="A68" s="17" t="n">
-        <v>6</v>
-      </c>
-      <c r="B68" s="18" t="inlineStr">
-        <is>
-          <t>HOMEASCOMM</t>
-        </is>
-      </c>
-      <c r="C68" s="18" t="inlineStr">
-        <is>
-          <t>SMeasure</t>
-        </is>
-      </c>
-      <c r="D68" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E68" s="18" t="inlineStr">
-        <is>
-          <t>Calibrate from MR. Must not hide intended A4.</t>
-        </is>
-      </c>
-      <c r="F68" s="17" t="inlineStr">
-        <is>
-          <t>Tune</t>
-        </is>
-      </c>
-      <c r="G68" s="18" t="inlineStr">
-        <is>
-          <t>4.1.5</t>
-        </is>
-      </c>
-      <c r="H68" s="18" t="inlineStr">
-        <is>
-          <t>Serving-cell RSRP above this value allows the UE to skip intra/inter/IRAT measurement.</t>
-        </is>
-      </c>
-      <c r="I68" s="18" t="inlineStr">
-        <is>
-          <t>LBFD-002018  ·  Mobility Management in Connected Mode Feature Parameter Description  ·  eRAN21.1 Issue 08  ·  §4.1.5</t>
-        </is>
-      </c>
-    </row>
-    <row r="69" ht="58" customHeight="1">
-      <c r="A69" s="17" t="n">
-        <v>7</v>
-      </c>
-      <c r="B69" s="18" t="inlineStr">
-        <is>
-          <t>INTRARATHOCOMM</t>
-        </is>
-      </c>
-      <c r="C69" s="18" t="inlineStr">
-        <is>
-          <t>InterFreqHoA1A2TrigQuan</t>
-        </is>
-      </c>
-      <c r="D69" s="19" t="inlineStr">
-        <is>
-          <t>RSRP</t>
-        </is>
-      </c>
-      <c r="E69" s="18" t="inlineStr">
-        <is>
-          <t>Recommended trigger quantity.</t>
-        </is>
-      </c>
-      <c r="F69" s="17" t="inlineStr">
-        <is>
-          <t>Tune</t>
-        </is>
-      </c>
-      <c r="G69" s="18" t="inlineStr">
-        <is>
-          <t>4.1.4</t>
-        </is>
-      </c>
-      <c r="H69" s="18" t="inlineStr">
-        <is>
-          <t>Quantity (RSRP / RSRQ / BOTH) used to trigger inter-frequency events A1 and A2.</t>
-        </is>
-      </c>
-      <c r="I69" s="18" t="inlineStr">
-        <is>
-          <t>LBFD-002018  ·  Mobility Management in Connected Mode Feature Parameter Description  ·  eRAN21.1 Issue 08  ·  §4.1.4</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" ht="58" customHeight="1">
-      <c r="A70" s="17" t="n">
-        <v>8</v>
-      </c>
-      <c r="B70" s="18" t="inlineStr">
-        <is>
-          <t>INTRARATHOCOMM</t>
-        </is>
-      </c>
-      <c r="C70" s="18" t="inlineStr">
-        <is>
-          <t>InterFreqHoA4TrigQuan</t>
-        </is>
-      </c>
-      <c r="D70" s="19" t="inlineStr">
-        <is>
-          <t>RSRP</t>
-        </is>
-      </c>
-      <c r="E70" s="18" t="inlineStr">
-        <is>
-          <t>Recommended. Reporting SAME_AS_TRIG_QUAN.</t>
-        </is>
-      </c>
-      <c r="F70" s="17" t="inlineStr">
-        <is>
-          <t>Tune</t>
-        </is>
-      </c>
-      <c r="G70" s="18" t="inlineStr">
-        <is>
-          <t>4.1.4</t>
-        </is>
-      </c>
-      <c r="H70" s="18" t="inlineStr">
-        <is>
-          <t>Quantity used to trigger inter-frequency event A4.</t>
-        </is>
-      </c>
-      <c r="I70" s="18" t="inlineStr">
-        <is>
-          <t>LBFD-002018  ·  Mobility Management in Connected Mode Feature Parameter Description  ·  eRAN21.1 Issue 08  ·  §4.1.4</t>
-        </is>
-      </c>
-    </row>
-    <row r="71" ht="58" customHeight="1">
-      <c r="A71" s="17" t="n">
-        <v>9</v>
-      </c>
-      <c r="B71" s="18" t="inlineStr">
-        <is>
-          <t>INTERFREQHOGROUP</t>
-        </is>
-      </c>
-      <c r="C71" s="18" t="inlineStr">
-        <is>
-          <t>InterFreqHoA1A2Hyst</t>
-        </is>
-      </c>
-      <c r="D71" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E71" s="18" t="inlineStr">
-        <is>
-          <t>Hys in A1/A2 formulas. Keep A1/A2 pair consistent.</t>
-        </is>
-      </c>
-      <c r="F71" s="17" t="inlineStr">
-        <is>
-          <t>Tune</t>
-        </is>
-      </c>
-      <c r="G71" s="18" t="inlineStr">
-        <is>
-          <t>Table 4-8</t>
-        </is>
-      </c>
-      <c r="H71" s="18" t="inlineStr">
-        <is>
-          <t>Hysteresis Hys applied to entering and leaving conditions of events A1 and A2.</t>
-        </is>
-      </c>
-      <c r="I71" s="18" t="inlineStr">
-        <is>
-          <t>LBFD-002018  ·  Mobility Management in Connected Mode Feature Parameter Description  ·  eRAN21.1 Issue 08  ·  Table 4-8</t>
         </is>
       </c>
     </row>
     <row r="72" ht="58" customHeight="1">
       <c r="A72" s="17" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="B72" s="18" t="inlineStr">
         <is>
-          <t>INTERFREQHOGROUP</t>
+          <t>EUTRANINTERNFREQ</t>
         </is>
       </c>
       <c r="C72" s="18" t="inlineStr">
         <is>
-          <t>InterFreqHoA1A2TimeToTrig</t>
+          <t>FREQ_MEAS_FLAG</t>
         </is>
       </c>
       <c r="D72" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>selected</t>
         </is>
       </c>
       <c r="E72" s="18" t="inlineStr">
         <is>
-          <t>TTT for A1/A2. QCI-specific optional.</t>
+          <t>Frequency must be measured. Silent no-HO if off.</t>
         </is>
       </c>
       <c r="F72" s="17" t="inlineStr">
         <is>
-          <t>Tune</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G72" s="18" t="inlineStr">
         <is>
-          <t>Table 4-8</t>
+          <t>4.1.4</t>
         </is>
       </c>
       <c r="H72" s="18" t="inlineStr">
         <is>
-          <t>Duration TimeToTrig that A1/A2 entering or leaving condition must hold.</t>
+          <t>Whether the UE is configured to measure this E-UTRAN frequency in connected mode.</t>
         </is>
       </c>
       <c r="I72" s="18" t="inlineStr">
         <is>
-          <t>LBFD-002018  ·  Mobility Management in Connected Mode Feature Parameter Description  ·  eRAN21.1 Issue 08  ·  Table 4-8</t>
+          <t>LBFD-002018  ·  Mobility Management in Connected Mode Feature Parameter Description  ·  eRAN21.1 Issue 08  ·  §4.1.4</t>
         </is>
       </c>
     </row>
     <row r="73" ht="58" customHeight="1">
       <c r="A73" s="17" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="B73" s="18" t="inlineStr">
         <is>
-          <t>INTERFREQHOGROUP</t>
+          <t>EUTRANINTERNFREQ</t>
         </is>
       </c>
       <c r="C73" s="18" t="inlineStr">
         <is>
-          <t>InterFreqHoA4Hyst</t>
+          <t>HO_TRG_FREQ_FORBID_MEAS_FLAG</t>
         </is>
       </c>
       <c r="D73" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>deselected</t>
         </is>
       </c>
       <c r="E73" s="18" t="inlineStr">
         <is>
-          <t>Hys in A4: Mn+Ofn+Ocn−Hys &gt; Thresh.</t>
+          <t>Must be off for required HO targets.</t>
         </is>
       </c>
       <c r="F73" s="17" t="inlineStr">
         <is>
-          <t>Tune</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G73" s="18" t="inlineStr">
         <is>
-          <t>Table 4-8</t>
+          <t>4.1.4</t>
         </is>
       </c>
       <c r="H73" s="18" t="inlineStr">
         <is>
-          <t>Hysteresis Hys in the event A4 formula.</t>
+          <t>If selected, this frequency is forbidden as a handover target even if measured.</t>
         </is>
       </c>
       <c r="I73" s="18" t="inlineStr">
         <is>
-          <t>LBFD-002018  ·  Mobility Management in Connected Mode Feature Parameter Description  ·  eRAN21.1 Issue 08  ·  Table 4-8</t>
+          <t>LBFD-002018  ·  Mobility Management in Connected Mode Feature Parameter Description  ·  eRAN21.1 Issue 08  ·  §4.1.4</t>
         </is>
       </c>
     </row>
     <row r="74" ht="58" customHeight="1">
       <c r="A74" s="17" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="B74" s="18" t="inlineStr">
         <is>
-          <t>INTERFREQHOGROUP</t>
+          <t>EUTRANINTERFREQNCELL</t>
         </is>
       </c>
       <c r="C74" s="18" t="inlineStr">
         <is>
-          <t>InterFreqHoA4TimeToTrig</t>
+          <t>NoHoFlag</t>
         </is>
       </c>
       <c r="D74" s="19" t="inlineStr">
         <is>
-          <t>not 5120 ms</t>
+          <t>PERMIT_HO</t>
         </is>
       </c>
       <c r="E74" s="18" t="inlineStr">
         <is>
-          <t>5120 ms disables FreqPri, CQI and service-based IFHO (eRAN21.1 Table 4-9).</t>
+          <t>Neighbour allowed as HO target.</t>
         </is>
       </c>
       <c r="F74" s="17" t="inlineStr">
@@ -5638,47 +5348,47 @@
       </c>
       <c r="G74" s="18" t="inlineStr">
         <is>
-          <t>Table 4-9</t>
+          <t>4.1.4</t>
         </is>
       </c>
       <c r="H74" s="18" t="inlineStr">
         <is>
-          <t>Duration TimeToTrig for event A4. 5120 ms is treated as disable for FreqPri / CQI / service IFHO.</t>
+          <t>Per-neighbour flag allowing or prohibiting handover to that cell.</t>
         </is>
       </c>
       <c r="I74" s="18" t="inlineStr">
         <is>
-          <t>LBFD-002018  ·  Mobility Management in Connected Mode Feature Parameter Description  ·  eRAN21.1 Issue 08  ·  Table 4-9</t>
+          <t>LBFD-002018  ·  Mobility Management in Connected Mode Feature Parameter Description  ·  eRAN21.1 Issue 08  ·  §4.1.4</t>
         </is>
       </c>
     </row>
     <row r="75" ht="58" customHeight="1">
       <c r="A75" s="17" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="B75" s="18" t="inlineStr">
         <is>
-          <t>INTRAFREQHOGROUP</t>
+          <t>CELLUEMEASCONTROLCFG</t>
         </is>
       </c>
       <c r="C75" s="18" t="inlineStr">
         <is>
-          <t>IntraFreqHoA3Offset</t>
+          <t>MaxNonIntraMeasObjNum</t>
         </is>
       </c>
       <c r="D75" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>≥ needed objects</t>
         </is>
       </c>
       <c r="E75" s="18" t="inlineStr">
         <is>
-          <t>Off in intra-frequency A3 formula.</t>
+          <t>Over cap: equal-priority objects drop at random.</t>
         </is>
       </c>
       <c r="F75" s="17" t="inlineStr">
         <is>
-          <t>Tune</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G75" s="18" t="inlineStr">
@@ -5688,42 +5398,42 @@
       </c>
       <c r="H75" s="18" t="inlineStr">
         <is>
-          <t>Offset Off added on the serving side of intra-frequency event A3.</t>
+          <t>Maximum number of non-intra-frequency measurement objects the eNodeB may deliver to a UE.</t>
         </is>
       </c>
       <c r="I75" s="18" t="inlineStr">
         <is>
-          <t>LBFD-002018  ·  Mobility Management in Connected Mode Feature Parameter Description  ·  eRAN21.1 Issue 08  ·  §4.1.4</t>
+          <t>LBFD-002018  ·  Mobility Management in Connected Mode Feature Parameter Description  ·  eRAN21.1 Issue 08  ·  Table 4-3</t>
         </is>
       </c>
     </row>
     <row r="76" ht="58" customHeight="1">
       <c r="A76" s="17" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="B76" s="18" t="inlineStr">
         <is>
-          <t>INTERFREQHOGROUP</t>
+          <t>CELLUEMEASCONTROLCFG</t>
         </is>
       </c>
       <c r="C76" s="18" t="inlineStr">
         <is>
-          <t>InterFreqHoA3Offset</t>
+          <t>MaxEutranFddMeasFreqNum</t>
         </is>
       </c>
       <c r="D76" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>≥ needed FDD freqs</t>
         </is>
       </c>
       <c r="E76" s="18" t="inlineStr">
         <is>
-          <t>Off in inter-frequency A3 formula.</t>
+          <t>Same random-drop risk for FDD.</t>
         </is>
       </c>
       <c r="F76" s="17" t="inlineStr">
         <is>
-          <t>Tune</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G76" s="18" t="inlineStr">
@@ -5733,27 +5443,27 @@
       </c>
       <c r="H76" s="18" t="inlineStr">
         <is>
-          <t>Offset Off added on the serving side of inter-frequency event A3.</t>
+          <t>Maximum number of neighbouring E-UTRAN FDD frequencies that can be delivered for measurement.</t>
         </is>
       </c>
       <c r="I76" s="18" t="inlineStr">
         <is>
-          <t>LBFD-002018  ·  Mobility Management in Connected Mode Feature Parameter Description  ·  eRAN21.1 Issue 08  ·  §4.1.4</t>
+          <t>LBFD-002018  ·  Mobility Management in Connected Mode Feature Parameter Description  ·  eRAN21.1 Issue 08  ·  Table 4-3</t>
         </is>
       </c>
     </row>
     <row r="77" ht="58" customHeight="1">
       <c r="A77" s="17" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="B77" s="18" t="inlineStr">
         <is>
-          <t>EUTRANINTERFREQNCELL</t>
+          <t>HOMEASCOMM</t>
         </is>
       </c>
       <c r="C77" s="18" t="inlineStr">
         <is>
-          <t>CellIndividualOffset</t>
+          <t>SMeasure</t>
         </is>
       </c>
       <c r="D77" s="19" t="inlineStr">
@@ -5763,7 +5473,7 @@
       </c>
       <c r="E77" s="18" t="inlineStr">
         <is>
-          <t>Ocn. Large CIO can mask RF overshoot.</t>
+          <t>Calibrate from MR. Must not hide intended A4.</t>
         </is>
       </c>
       <c r="F77" s="17" t="inlineStr">
@@ -5773,42 +5483,42 @@
       </c>
       <c r="G77" s="18" t="inlineStr">
         <is>
-          <t>4.1.4</t>
+          <t>4.1.5</t>
         </is>
       </c>
       <c r="H77" s="18" t="inlineStr">
         <is>
-          <t>Cell-specific offset Ocn (CIO) for the neighbouring cell in A3/A4/A5.</t>
+          <t>Serving-cell RSRP above this value allows the UE to skip intra/inter/IRAT measurement.</t>
         </is>
       </c>
       <c r="I77" s="18" t="inlineStr">
         <is>
-          <t>LBFD-002018  ·  Mobility Management in Connected Mode Feature Parameter Description  ·  eRAN21.1 Issue 08  ·  §4.1.4</t>
+          <t>LBFD-002018  ·  Mobility Management in Connected Mode Feature Parameter Description  ·  eRAN21.1 Issue 08  ·  §4.1.5</t>
         </is>
       </c>
     </row>
     <row r="78" ht="58" customHeight="1">
       <c r="A78" s="17" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B78" s="18" t="inlineStr">
         <is>
-          <t>EUTRANINTERNFREQ</t>
+          <t>INTRARATHOCOMM</t>
         </is>
       </c>
       <c r="C78" s="18" t="inlineStr">
         <is>
-          <t>QoffsetFreq</t>
+          <t>InterFreqHoA1A2TrigQuan</t>
         </is>
       </c>
       <c r="D78" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>RSRP</t>
         </is>
       </c>
       <c r="E78" s="18" t="inlineStr">
         <is>
-          <t>Ofn / connected frequency offset.</t>
+          <t>Recommended trigger quantity.</t>
         </is>
       </c>
       <c r="F78" s="17" t="inlineStr">
@@ -5823,7 +5533,7 @@
       </c>
       <c r="H78" s="18" t="inlineStr">
         <is>
-          <t>Frequency-specific offset Ofn for the neighbouring frequency.</t>
+          <t>Quantity (RSRP / RSRQ / BOTH) used to trigger inter-frequency events A1 and A2.</t>
         </is>
       </c>
       <c r="I78" s="18" t="inlineStr">
@@ -5834,26 +5544,26 @@
     </row>
     <row r="79" ht="58" customHeight="1">
       <c r="A79" s="17" t="n">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="B79" s="18" t="inlineStr">
         <is>
-          <t>CELLHOPARACFG</t>
+          <t>INTRARATHOCOMM</t>
         </is>
       </c>
       <c r="C79" s="18" t="inlineStr">
         <is>
-          <t>EutranFilterCoeffRsrp</t>
+          <t>InterFreqHoA4TrigQuan</t>
         </is>
       </c>
       <c r="D79" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>RSRP</t>
         </is>
       </c>
       <c r="E79" s="18" t="inlineStr">
         <is>
-          <t>L3 RSRP filter. Over-smooth delays coverage rescue.</t>
+          <t>Recommended. Reporting SAME_AS_TRIG_QUAN.</t>
         </is>
       </c>
       <c r="F79" s="17" t="inlineStr">
@@ -5868,7 +5578,7 @@
       </c>
       <c r="H79" s="18" t="inlineStr">
         <is>
-          <t>Layer-3 filter coefficient applied to RSRP before event evaluation.</t>
+          <t>Quantity used to trigger inter-frequency event A4.</t>
         </is>
       </c>
       <c r="I79" s="18" t="inlineStr">
@@ -5879,26 +5589,26 @@
     </row>
     <row r="80" ht="58" customHeight="1">
       <c r="A80" s="17" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="B80" s="18" t="inlineStr">
         <is>
-          <t>CELLALGOSWITCH</t>
+          <t>INTERFREQHOGROUP</t>
         </is>
       </c>
       <c r="C80" s="18" t="inlineStr">
         <is>
-          <t>MEAS_OBJ_PREEMPT_SW</t>
+          <t>InterFreqHoA1A2Hyst</t>
         </is>
       </c>
       <c r="D80" s="19" t="inlineStr">
         <is>
-          <t>as designed</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E80" s="18" t="inlineStr">
         <is>
-          <t>Higher-priority algorithm can take limited UE gap capability.</t>
+          <t>Hys in A1/A2 formulas. Keep A1/A2 pair consistent.</t>
         </is>
       </c>
       <c r="F80" s="17" t="inlineStr">
@@ -5908,42 +5618,42 @@
       </c>
       <c r="G80" s="18" t="inlineStr">
         <is>
-          <t>Table 4-4</t>
+          <t>Table 4-8</t>
         </is>
       </c>
       <c r="H80" s="18" t="inlineStr">
         <is>
-          <t>Allows a higher-priority measurement algorithm to preempt gap resources of a limited-capability UE.</t>
+          <t>Hysteresis Hys applied to entering and leaving conditions of events A1 and A2.</t>
         </is>
       </c>
       <c r="I80" s="18" t="inlineStr">
         <is>
-          <t>LBFD-002018  ·  Mobility Management in Connected Mode Feature Parameter Description  ·  eRAN21.1 Issue 08  ·  Table 4-4</t>
+          <t>LBFD-002018  ·  Mobility Management in Connected Mode Feature Parameter Description  ·  eRAN21.1 Issue 08  ·  Table 4-8</t>
         </is>
       </c>
     </row>
     <row r="81" ht="58" customHeight="1">
       <c r="A81" s="17" t="n">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="B81" s="18" t="inlineStr">
         <is>
-          <t>ENODEBALGOSWITCH</t>
+          <t>INTERFREQHOGROUP</t>
         </is>
       </c>
       <c r="C81" s="18" t="inlineStr">
         <is>
-          <t>AutoGapSwitch</t>
+          <t>InterFreqHoA1A2TimeToTrig</t>
         </is>
       </c>
       <c r="D81" s="19" t="inlineStr">
         <is>
-          <t>as designed</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E81" s="18" t="inlineStr">
         <is>
-          <t>Gap pattern cost on DL TTI / VoLTE.</t>
+          <t>TTT for A1/A2. QCI-specific optional.</t>
         </is>
       </c>
       <c r="F81" s="17" t="inlineStr">
@@ -5953,113 +5663,524 @@
       </c>
       <c r="G81" s="18" t="inlineStr">
         <is>
-          <t>4.1.4</t>
+          <t>Table 4-8</t>
         </is>
       </c>
       <c r="H81" s="18" t="inlineStr">
         <is>
-          <t>Controls automatic delivery of measurement gap patterns for inter-frequency / IRAT measurement.</t>
+          <t>Duration TimeToTrig that A1/A2 entering or leaving condition must hold.</t>
         </is>
       </c>
       <c r="I81" s="18" t="inlineStr">
         <is>
-          <t>LBFD-002018  ·  Mobility Management in Connected Mode Feature Parameter Description  ·  eRAN21.1 Issue 08  ·  §4.1.4</t>
+          <t>LBFD-002018  ·  Mobility Management in Connected Mode Feature Parameter Description  ·  eRAN21.1 Issue 08  ·  Table 4-8</t>
         </is>
       </c>
     </row>
     <row r="82" ht="58" customHeight="1">
       <c r="A82" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="B82" s="18" t="inlineStr">
+        <is>
+          <t>INTERFREQHOGROUP</t>
+        </is>
+      </c>
+      <c r="C82" s="18" t="inlineStr">
+        <is>
+          <t>InterFreqHoA4Hyst</t>
+        </is>
+      </c>
+      <c r="D82" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E82" s="18" t="inlineStr">
+        <is>
+          <t>Hys in A4: Mn+Ofn+Ocn−Hys &gt; Thresh.</t>
+        </is>
+      </c>
+      <c r="F82" s="17" t="inlineStr">
+        <is>
+          <t>Tune</t>
+        </is>
+      </c>
+      <c r="G82" s="18" t="inlineStr">
+        <is>
+          <t>Table 4-8</t>
+        </is>
+      </c>
+      <c r="H82" s="18" t="inlineStr">
+        <is>
+          <t>Hysteresis Hys in the event A4 formula.</t>
+        </is>
+      </c>
+      <c r="I82" s="18" t="inlineStr">
+        <is>
+          <t>LBFD-002018  ·  Mobility Management in Connected Mode Feature Parameter Description  ·  eRAN21.1 Issue 08  ·  Table 4-8</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="58" customHeight="1">
+      <c r="A83" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="B83" s="18" t="inlineStr">
+        <is>
+          <t>INTERFREQHOGROUP</t>
+        </is>
+      </c>
+      <c r="C83" s="18" t="inlineStr">
+        <is>
+          <t>InterFreqHoA4TimeToTrig</t>
+        </is>
+      </c>
+      <c r="D83" s="19" t="inlineStr">
+        <is>
+          <t>not 5120 ms</t>
+        </is>
+      </c>
+      <c r="E83" s="18" t="inlineStr">
+        <is>
+          <t>5120 ms disables FreqPri, CQI and service-based IFHO (eRAN21.1 Table 4-9).</t>
+        </is>
+      </c>
+      <c r="F83" s="17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G83" s="18" t="inlineStr">
+        <is>
+          <t>Table 4-9</t>
+        </is>
+      </c>
+      <c r="H83" s="18" t="inlineStr">
+        <is>
+          <t>Duration TimeToTrig for event A4. 5120 ms is treated as disable for FreqPri / CQI / service IFHO.</t>
+        </is>
+      </c>
+      <c r="I83" s="18" t="inlineStr">
+        <is>
+          <t>LBFD-002018  ·  Mobility Management in Connected Mode Feature Parameter Description  ·  eRAN21.1 Issue 08  ·  Table 4-9</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="58" customHeight="1">
+      <c r="A84" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="B84" s="18" t="inlineStr">
+        <is>
+          <t>INTRAFREQHOGROUP</t>
+        </is>
+      </c>
+      <c r="C84" s="18" t="inlineStr">
+        <is>
+          <t>IntraFreqHoA3Offset</t>
+        </is>
+      </c>
+      <c r="D84" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E84" s="18" t="inlineStr">
+        <is>
+          <t>Off in intra-frequency A3 formula.</t>
+        </is>
+      </c>
+      <c r="F84" s="17" t="inlineStr">
+        <is>
+          <t>Tune</t>
+        </is>
+      </c>
+      <c r="G84" s="18" t="inlineStr">
+        <is>
+          <t>4.1.4</t>
+        </is>
+      </c>
+      <c r="H84" s="18" t="inlineStr">
+        <is>
+          <t>Offset Off added on the serving side of intra-frequency event A3.</t>
+        </is>
+      </c>
+      <c r="I84" s="18" t="inlineStr">
+        <is>
+          <t>LBFD-002018  ·  Mobility Management in Connected Mode Feature Parameter Description  ·  eRAN21.1 Issue 08  ·  §4.1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="58" customHeight="1">
+      <c r="A85" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="B85" s="18" t="inlineStr">
+        <is>
+          <t>INTERFREQHOGROUP</t>
+        </is>
+      </c>
+      <c r="C85" s="18" t="inlineStr">
+        <is>
+          <t>InterFreqHoA3Offset</t>
+        </is>
+      </c>
+      <c r="D85" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E85" s="18" t="inlineStr">
+        <is>
+          <t>Off in inter-frequency A3 formula.</t>
+        </is>
+      </c>
+      <c r="F85" s="17" t="inlineStr">
+        <is>
+          <t>Tune</t>
+        </is>
+      </c>
+      <c r="G85" s="18" t="inlineStr">
+        <is>
+          <t>4.1.4</t>
+        </is>
+      </c>
+      <c r="H85" s="18" t="inlineStr">
+        <is>
+          <t>Offset Off added on the serving side of inter-frequency event A3.</t>
+        </is>
+      </c>
+      <c r="I85" s="18" t="inlineStr">
+        <is>
+          <t>LBFD-002018  ·  Mobility Management in Connected Mode Feature Parameter Description  ·  eRAN21.1 Issue 08  ·  §4.1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="58" customHeight="1">
+      <c r="A86" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="B86" s="18" t="inlineStr">
+        <is>
+          <t>EUTRANINTERFREQNCELL</t>
+        </is>
+      </c>
+      <c r="C86" s="18" t="inlineStr">
+        <is>
+          <t>CellIndividualOffset</t>
+        </is>
+      </c>
+      <c r="D86" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E86" s="18" t="inlineStr">
+        <is>
+          <t>Ocn. Large CIO can mask RF overshoot.</t>
+        </is>
+      </c>
+      <c r="F86" s="17" t="inlineStr">
+        <is>
+          <t>Tune</t>
+        </is>
+      </c>
+      <c r="G86" s="18" t="inlineStr">
+        <is>
+          <t>4.1.4</t>
+        </is>
+      </c>
+      <c r="H86" s="18" t="inlineStr">
+        <is>
+          <t>Cell-specific offset Ocn (CIO) for the neighbouring cell in A3/A4/A5.</t>
+        </is>
+      </c>
+      <c r="I86" s="18" t="inlineStr">
+        <is>
+          <t>LBFD-002018  ·  Mobility Management in Connected Mode Feature Parameter Description  ·  eRAN21.1 Issue 08  ·  §4.1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="58" customHeight="1">
+      <c r="A87" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B87" s="18" t="inlineStr">
+        <is>
+          <t>EUTRANINTERNFREQ</t>
+        </is>
+      </c>
+      <c r="C87" s="18" t="inlineStr">
+        <is>
+          <t>QoffsetFreq</t>
+        </is>
+      </c>
+      <c r="D87" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E87" s="18" t="inlineStr">
+        <is>
+          <t>Ofn / connected frequency offset.</t>
+        </is>
+      </c>
+      <c r="F87" s="17" t="inlineStr">
+        <is>
+          <t>Tune</t>
+        </is>
+      </c>
+      <c r="G87" s="18" t="inlineStr">
+        <is>
+          <t>4.1.4</t>
+        </is>
+      </c>
+      <c r="H87" s="18" t="inlineStr">
+        <is>
+          <t>Frequency-specific offset Ofn for the neighbouring frequency.</t>
+        </is>
+      </c>
+      <c r="I87" s="18" t="inlineStr">
+        <is>
+          <t>LBFD-002018  ·  Mobility Management in Connected Mode Feature Parameter Description  ·  eRAN21.1 Issue 08  ·  §4.1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="58" customHeight="1">
+      <c r="A88" s="17" t="n">
+        <v>17</v>
+      </c>
+      <c r="B88" s="18" t="inlineStr">
+        <is>
+          <t>CELLHOPARACFG</t>
+        </is>
+      </c>
+      <c r="C88" s="18" t="inlineStr">
+        <is>
+          <t>EutranFilterCoeffRsrp</t>
+        </is>
+      </c>
+      <c r="D88" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E88" s="18" t="inlineStr">
+        <is>
+          <t>L3 RSRP filter. Over-smooth delays coverage rescue.</t>
+        </is>
+      </c>
+      <c r="F88" s="17" t="inlineStr">
+        <is>
+          <t>Tune</t>
+        </is>
+      </c>
+      <c r="G88" s="18" t="inlineStr">
+        <is>
+          <t>4.1.4</t>
+        </is>
+      </c>
+      <c r="H88" s="18" t="inlineStr">
+        <is>
+          <t>Layer-3 filter coefficient applied to RSRP before event evaluation.</t>
+        </is>
+      </c>
+      <c r="I88" s="18" t="inlineStr">
+        <is>
+          <t>LBFD-002018  ·  Mobility Management in Connected Mode Feature Parameter Description  ·  eRAN21.1 Issue 08  ·  §4.1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="58" customHeight="1">
+      <c r="A89" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="B89" s="18" t="inlineStr">
+        <is>
+          <t>CELLALGOSWITCH</t>
+        </is>
+      </c>
+      <c r="C89" s="18" t="inlineStr">
+        <is>
+          <t>MEAS_OBJ_PREEMPT_SW</t>
+        </is>
+      </c>
+      <c r="D89" s="19" t="inlineStr">
+        <is>
+          <t>as designed</t>
+        </is>
+      </c>
+      <c r="E89" s="18" t="inlineStr">
+        <is>
+          <t>Higher-priority algorithm can take limited UE gap capability.</t>
+        </is>
+      </c>
+      <c r="F89" s="17" t="inlineStr">
+        <is>
+          <t>Tune</t>
+        </is>
+      </c>
+      <c r="G89" s="18" t="inlineStr">
+        <is>
+          <t>Table 4-4</t>
+        </is>
+      </c>
+      <c r="H89" s="18" t="inlineStr">
+        <is>
+          <t>Allows a higher-priority measurement algorithm to preempt gap resources of a limited-capability UE.</t>
+        </is>
+      </c>
+      <c r="I89" s="18" t="inlineStr">
+        <is>
+          <t>LBFD-002018  ·  Mobility Management in Connected Mode Feature Parameter Description  ·  eRAN21.1 Issue 08  ·  Table 4-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="58" customHeight="1">
+      <c r="A90" s="17" t="n">
+        <v>19</v>
+      </c>
+      <c r="B90" s="18" t="inlineStr">
+        <is>
+          <t>ENODEBALGOSWITCH</t>
+        </is>
+      </c>
+      <c r="C90" s="18" t="inlineStr">
+        <is>
+          <t>AutoGapSwitch</t>
+        </is>
+      </c>
+      <c r="D90" s="19" t="inlineStr">
+        <is>
+          <t>as designed</t>
+        </is>
+      </c>
+      <c r="E90" s="18" t="inlineStr">
+        <is>
+          <t>Gap pattern cost on DL TTI / VoLTE.</t>
+        </is>
+      </c>
+      <c r="F90" s="17" t="inlineStr">
+        <is>
+          <t>Tune</t>
+        </is>
+      </c>
+      <c r="G90" s="18" t="inlineStr">
+        <is>
+          <t>4.1.4</t>
+        </is>
+      </c>
+      <c r="H90" s="18" t="inlineStr">
+        <is>
+          <t>Controls automatic delivery of measurement gap patterns for inter-frequency / IRAT measurement.</t>
+        </is>
+      </c>
+      <c r="I90" s="18" t="inlineStr">
+        <is>
+          <t>LBFD-002018  ·  Mobility Management in Connected Mode Feature Parameter Description  ·  eRAN21.1 Issue 08  ·  §4.1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="58" customHeight="1">
+      <c r="A91" s="17" t="n">
         <v>20</v>
       </c>
-      <c r="B82" s="18" t="inlineStr">
+      <c r="B91" s="18" t="inlineStr">
         <is>
           <t>CELLQCIPARA</t>
         </is>
       </c>
-      <c r="C82" s="18" t="inlineStr">
+      <c r="C91" s="18" t="inlineStr">
         <is>
           <t>QciPriorityForHo</t>
         </is>
       </c>
-      <c r="D82" s="19" t="inlineStr">
+      <c r="D91" s="19" t="inlineStr">
         <is>
           <t>see default map</t>
         </is>
       </c>
-      <c r="E82" s="18" t="inlineStr">
+      <c r="E91" s="18" t="inlineStr">
         <is>
           <t>FDD default: QCI5=1, QCI1=2, QCI3=3, QCI2=4, QCI4=5, QCI6=6, QCI7=7, QCI8=8, QCI9=9. Smaller = higher priority.</t>
         </is>
       </c>
-      <c r="F82" s="17" t="inlineStr">
+      <c r="F91" s="17" t="inlineStr">
         <is>
           <t>Tune</t>
         </is>
       </c>
-      <c r="G82" s="18" t="inlineStr">
+      <c r="G91" s="18" t="inlineStr">
         <is>
           <t>Table 4-10</t>
         </is>
       </c>
-      <c r="H82" s="18" t="inlineStr">
+      <c r="H91" s="18" t="inlineStr">
         <is>
           <t>Priority used when several QCIs run together so the eNodeB knows which QCI’s HO parameters to deliver.</t>
         </is>
       </c>
-      <c r="I82" s="18" t="inlineStr">
+      <c r="I91" s="18" t="inlineStr">
         <is>
           <t>LBFD-002018  ·  Mobility Management in Connected Mode Feature Parameter Description  ·  eRAN21.1 Issue 08  ·  Table 4-10</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="47">
+  <mergeCells count="53">
     <mergeCell ref="A7:I7"/>
+    <mergeCell ref="A65:I65"/>
     <mergeCell ref="A41:I41"/>
+    <mergeCell ref="A54:I54"/>
     <mergeCell ref="A37:I37"/>
     <mergeCell ref="A46:I46"/>
-    <mergeCell ref="A56:I56"/>
+    <mergeCell ref="D61:I61"/>
     <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A55:I55"/>
     <mergeCell ref="A12:I12"/>
     <mergeCell ref="A50:I50"/>
     <mergeCell ref="A26:I26"/>
     <mergeCell ref="A21:I21"/>
-    <mergeCell ref="D53:I53"/>
+    <mergeCell ref="A57:I57"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A33:I33"/>
+    <mergeCell ref="A47:I47"/>
+    <mergeCell ref="D62:I62"/>
     <mergeCell ref="A14:I14"/>
     <mergeCell ref="A17:I17"/>
     <mergeCell ref="A23:I23"/>
-    <mergeCell ref="A53:C53"/>
+    <mergeCell ref="A62:C62"/>
     <mergeCell ref="A29:C29"/>
     <mergeCell ref="A35:I35"/>
     <mergeCell ref="D30:I30"/>
     <mergeCell ref="A38:I38"/>
-    <mergeCell ref="A52:C52"/>
+    <mergeCell ref="A52:I52"/>
     <mergeCell ref="A43:I43"/>
-    <mergeCell ref="D51:I51"/>
     <mergeCell ref="A19:I19"/>
+    <mergeCell ref="A63:C63"/>
     <mergeCell ref="A10:I10"/>
     <mergeCell ref="A28:I28"/>
     <mergeCell ref="D29:I29"/>
     <mergeCell ref="A13:I13"/>
     <mergeCell ref="A31:C31"/>
-    <mergeCell ref="D54:I54"/>
+    <mergeCell ref="A44:I44"/>
+    <mergeCell ref="A40:I40"/>
     <mergeCell ref="A9:I9"/>
+    <mergeCell ref="A67:I67"/>
     <mergeCell ref="A30:C30"/>
-    <mergeCell ref="A58:I58"/>
-    <mergeCell ref="A39:I39"/>
+    <mergeCell ref="D60:I60"/>
     <mergeCell ref="A48:I48"/>
     <mergeCell ref="A24:I24"/>
-    <mergeCell ref="A51:C51"/>
     <mergeCell ref="A15:I15"/>
+    <mergeCell ref="A59:I59"/>
+    <mergeCell ref="A60:C60"/>
+    <mergeCell ref="D63:I63"/>
     <mergeCell ref="A11:I11"/>
-    <mergeCell ref="A60:I60"/>
+    <mergeCell ref="A61:C61"/>
     <mergeCell ref="D31:I31"/>
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A45:I45"/>
-    <mergeCell ref="D52:I52"/>
-    <mergeCell ref="A54:C54"/>
+    <mergeCell ref="A69:I69"/>
     <mergeCell ref="A16:I16"/>
   </mergeCells>
   <hyperlinks>
@@ -6236,7 +6357,7 @@
       <c r="H20" s="29" t="n"/>
       <c r="I20" s="29" t="n"/>
     </row>
-    <row r="21" ht="110" customHeight="1">
+    <row r="21" ht="144" customHeight="1">
       <c r="A21" s="30" t="inlineStr">
         <is>
           <t>A3-based IFHO A2:  A3InterFreqHoA2ThdRsrp  +  operator/QCI offset (eNBCnOpQciRsvdPara)   when InterFreqHoEventType = EventA3
@@ -6244,7 +6365,9 @@
 IRAT A2:  InterRatHoA2ThdRsrp / Rsrq. Further split UTRAN vs GERAN if an A2 offset is set per RAT.
 Blind A2:  CellHoParaCfg.BlindHoA1A2ThdRsrp / Rsrq
 If measurement A2 threshold ≤ blind A2, the eNodeB delivers only blind A2.
-A4/A5 target threshold must be better than this coverage A2, or the UE ping-pongs back.</t>
+A4/A5 target threshold must be better than this coverage A2 (higher RSRP requirement: A4_thd &gt; A2_thd), or the UE ping-pongs back.
+Example (not a design): A3-based A2 base = −110 dBm, operator/QCI offset = +4 dB → −106 dBm. Clamp MAX(−140, MIN(−43, −106)) = −106 dBm. That −106 dBm is the A2 the UE uses.
+Example ping-pong check: coverage A2 = −110 dBm, so A4 must be higher than −110 dBm (for example A4 = −105 dBm). Unsafe: A2 = −100 and A4 = −110 lets a neighbour at −107 dBm HO, then A2 fires on the new cell (−107 + 2 = −105 &lt; −100).</t>
         </is>
       </c>
       <c r="B21" s="29" t="n"/>
@@ -6288,7 +6411,7 @@
       <c r="H27" s="14" t="n"/>
       <c r="I27" s="14" t="n"/>
     </row>
-    <row r="28" ht="42" customHeight="1">
+    <row r="28" ht="36" customHeight="1">
       <c r="A28" s="15" t="inlineStr">
         <is>
           <t>ENODEBALGOSWITCH HoAlgoSwitch IntraFreqCoverHoSwitch = ON. IntraFreqHoA3TrigQuan = RSRP (default).</t>
@@ -6307,7 +6430,7 @@
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="28" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Calculation</t>
+          <t xml:space="preserve">  Calculation + example (not a design)</t>
         </is>
       </c>
       <c r="B30" s="29" t="n"/>
@@ -6319,10 +6442,13 @@
       <c r="H30" s="29" t="n"/>
       <c r="I30" s="29" t="n"/>
     </row>
-    <row r="31" ht="42" customHeight="1">
+    <row r="31" ht="80" customHeight="1">
       <c r="A31" s="30" t="inlineStr">
         <is>
-          <t>A3 enter: Mn + Ofn + Ocn − Hys &gt; Ms + Ofs + Ocs + IntraFreqHoA3Offset, true for IntraFreqHoA3TimeToTrig.</t>
+          <t>A3 enter: Mn + Ofn + Ocn − Hys &gt; Ms + Ofs + Ocs + IntraFreqHoA3Offset, true for IntraFreqHoA3TimeToTrig.
+Example: Ms = −95 dBm, Mn = −90 dBm, Hys = 2 dB, all offsets 0 except Off = 2 dB.
+Left = −90 − 2 = −92.  Right = −95 + 2 = −93.  −92 &gt; −93 → ENTER. Neighbour is 3 dB stronger, offset asks for 2 dB, hysteresis 2 dB, so A3 just passes.
+If IntraFreqHoA3Offset = 6 dB: Right = −89.  −92 &gt; −89 → NO. Increase Off to stop early intra-frequency HO.</t>
         </is>
       </c>
       <c r="B31" s="29" t="n"/>
@@ -6407,7 +6533,7 @@
       <c r="H36" s="32" t="n"/>
       <c r="I36" s="32" t="n"/>
     </row>
-    <row r="37" ht="42" customHeight="1">
+    <row r="37" ht="36" customHeight="1">
       <c r="A37" s="33" t="inlineStr">
         <is>
           <t>Chapter 4 NRT and CIO must be valid. License: none.</t>
@@ -6454,7 +6580,7 @@
       <c r="H43" s="14" t="n"/>
       <c r="I43" s="14" t="n"/>
     </row>
-    <row r="44" ht="98" customHeight="1">
+    <row r="44" ht="80" customHeight="1">
       <c r="A44" s="15" t="inlineStr">
         <is>
           <t>CELLHOPARACFG CellHoAlgoSwitch InterFreqCoverHoSwitch = ON.
@@ -6476,7 +6602,7 @@
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="28" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Calculation</t>
+          <t xml:space="preserve">  Calculation + example (not a design)</t>
         </is>
       </c>
       <c r="B46" s="29" t="n"/>
@@ -6488,12 +6614,15 @@
       <c r="H46" s="29" t="n"/>
       <c r="I46" s="29" t="n"/>
     </row>
-    <row r="47" ht="84" customHeight="1">
+    <row r="47" ht="112" customHeight="1">
       <c r="A47" s="30" t="inlineStr">
         <is>
           <t>Start meas: A2  Ms + Hys &lt; A2_thd  for TTT. Stop: A1  Ms − Hys &gt; A1_thd.
 Target A3: relative. Target A4: Mn+Ofn+Ocn−Hys &gt; InterFreqHoA4ThdRSRP. Target A5: serving &lt; Th1 AND neighbour &gt; Th2.
-Preferential blind: same A2 as measurement IFHO, but HO instead of meas. Emergency blind: worse A2, policy = redirection.</t>
+Preferential blind: same A2 as measurement IFHO, but HO instead of meas. Emergency blind: worse A2, policy = redirection.
+Example A2 start: A2_thd = −110 dBm, Hys = 2 dB, Ms = −115 dBm.  −115 + 2 = −113 &lt; −110 → start inter-frequency measurement.
+Example A1 stop: A1_thd = −104 dBm (a few dB above A2 −110), Ms = −95 dBm.  −95 − 2 = −97 &gt; −104 → stop measurement, serving recovered. If Ms is still −108: −108 − 2 = −110 &gt; −104? NO — measurement continues.
+Example A4 target: A4 = −105 dBm, Mn = −90 dBm, Hys = 2.  −92 &gt; −105 → HO. Keep A4 (−105) higher than A2 (−110) so a just-good target is not immediately A2-poor.</t>
         </is>
       </c>
       <c r="B47" s="29" t="n"/>
@@ -6593,7 +6722,7 @@
       <c r="H53" s="32" t="n"/>
       <c r="I53" s="32" t="n"/>
     </row>
-    <row r="54" ht="42" customHeight="1">
+    <row r="54" ht="36" customHeight="1">
       <c r="A54" s="33" t="inlineStr">
         <is>
           <t>Ch.4 flags and object cap. A4/A5 thd better than this A2. Book MML examples −85/−87 dBm are not design values.</t>
@@ -6640,7 +6769,7 @@
       <c r="H60" s="14" t="n"/>
       <c r="I60" s="14" t="n"/>
     </row>
-    <row r="61" ht="42" customHeight="1">
+    <row r="61" ht="36" customHeight="1">
       <c r="A61" s="15" t="inlineStr">
         <is>
           <t>UtranPsHoSwitch and/or UtranRedirectSwitch = ON. InterRatHoA1A2TrigQuan = RSRP recommended.</t>
@@ -6659,7 +6788,7 @@
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="28" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Calculation</t>
+          <t xml:space="preserve">  Calculation + example (not a design)</t>
         </is>
       </c>
       <c r="B63" s="29" t="n"/>
@@ -6671,10 +6800,13 @@
       <c r="H63" s="29" t="n"/>
       <c r="I63" s="29" t="n"/>
     </row>
-    <row r="64" ht="42" customHeight="1">
+    <row r="64" ht="80" customHeight="1">
       <c r="A64" s="30" t="inlineStr">
         <is>
-          <t>B1: Mn + Ofn − Hys &gt; B1_thd. B2: serving A2-style Th1 AND B1-style Th2.</t>
+          <t>B1: Mn + Ofn − Hys &gt; B1_thd. Example: IRAT Mn = −92, Ofn = 0, Hys = 2, B1_thd = −100.  −94 &gt; −100 → ENTER.
+B2: serving A2-style Th1 AND B1-style Th2. Example Th1 = −110, Th2 = −100, Ms = −115, Mn = −92, Hys = 2.
+     Serving: −115 + 2 = −113 &lt; −110 YES. Neighbour: −94 &gt; −100 YES → ENTER. If Ms = −95, serving −93 &lt; −110? NO — B2 does not enter.
+IRAT offload TTT must be &lt; 3 s or the 3 s meas stop kills the report.</t>
         </is>
       </c>
       <c r="B64" s="29" t="n"/>
@@ -6756,7 +6888,7 @@
       <c r="H72" s="14" t="n"/>
       <c r="I72" s="14" t="n"/>
     </row>
-    <row r="73" ht="42" customHeight="1">
+    <row r="73" ht="36" customHeight="1">
       <c r="A73" s="15" t="inlineStr">
         <is>
           <t>GeranRedirectSwitch = ON. Smaller B1 TTT toward UTRAN than GERAN makes UTRAN more likely given the same RF.</t>
@@ -6841,7 +6973,7 @@
       <c r="H81" s="14" t="n"/>
       <c r="I81" s="14" t="n"/>
     </row>
-    <row r="82" ht="42" customHeight="1">
+    <row r="82" ht="36" customHeight="1">
       <c r="A82" s="15" t="inlineStr">
         <is>
           <t>CELLALGOSWITCH FreqLayerSwitch UtranFreqLayerMeasSwitch and/or UtranFreqLayerBlindSwitch = ON. UTRANNFREQ CsPriority / PsPriority set. Priority_0 = do not use that frequency for that service.</t>
@@ -6872,7 +7004,7 @@
       <c r="H84" s="32" t="n"/>
       <c r="I84" s="32" t="n"/>
     </row>
-    <row r="85" ht="42" customHeight="1">
+    <row r="85" ht="36" customHeight="1">
       <c r="A85" s="33" t="inlineStr">
         <is>
           <t>Needs §5.4 coverage IRAT to UTRAN. Voice vs data RAT steering: SrvccRatSteeringSwitch / PsRatSteeringSwitch. RatLayerSwitch is legacy — not recommended.</t>
@@ -8184,7 +8316,7 @@
       <c r="H18" s="32" t="n"/>
       <c r="I18" s="32" t="n"/>
     </row>
-    <row r="19" ht="110" customHeight="1">
+    <row r="19" ht="80" customHeight="1">
       <c r="A19" s="33" t="inlineStr">
         <is>
           <t>Chapter 4 object cap and A4 TTT ≠ 5120 ms.
@@ -8227,7 +8359,7 @@
       <c r="H24" s="14" t="n"/>
       <c r="I24" s="14" t="n"/>
     </row>
-    <row r="25" ht="42" customHeight="1">
+    <row r="25" ht="36" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
         <is>
           <t>HoAlgoSwitch ServiceBasedInterFreqHoSwitch = ON  AND  CELLALGOSWITCH SrvBasedInterFreqHoSw = ON. CNOPERATORQCIPARA binds QCI to ServiceIfHoCfgGroup. InterFreqHoState = PERMIT_HO.</t>
@@ -8246,7 +8378,7 @@
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="28" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Calculation</t>
+          <t xml:space="preserve">  Calculation + example (not a design)</t>
         </is>
       </c>
       <c r="B27" s="29" t="n"/>
@@ -8258,13 +8390,15 @@
       <c r="H27" s="29" t="n"/>
       <c r="I27" s="29" t="n"/>
     </row>
-    <row r="28" ht="110" customHeight="1">
+    <row r="28" ht="128" customHeight="1">
       <c r="A28" s="30" t="inlineStr">
         <is>
           <t>Target event A4. Threshold = InterFreqLoadBasedHoA4ThdRSRP + QCI/operator offset (same A4 pool as FreqPri in many versions).
 Enter: Mn + Ofn + Ocn − Hys &gt; that threshold, for InterFreqHoA4TimeToTrig.
+Example: base A4 = −105 dBm, QCI offset = +3 dB → used A4 = −102 dBm. Mn = −90, Hys = 2.  −92 &gt; −102 → ENTER.
+If coverage A2 is −110 dBm, used A4 −102 dBm is higher than A2, so the UE is not coverage-measured out of the new cell at once.
 ServiceBasedMultiFreqHoSwitch ON: for CA-incapable UEs, pick high priority + high BW + light load. CA-capable UEs are then not service-HO’d (use CA smart selection instead).
-Light load: UL-sync UE count &lt; serving MlbUeNumThd + offset, or neighbour load unknown. Neighbour must send X2 load (YES).
+Light-load example: serving MlbUeNumThd = 40, offset = 5. Neighbour UL-sync UEs = 30.  30 &lt; 40+5 → treated as light load.
 ServBasedHoBackSwitch allows return to the source frequency on the next service HO.</t>
         </is>
       </c>
@@ -8374,7 +8508,7 @@
       <c r="H37" s="14" t="n"/>
       <c r="I37" s="14" t="n"/>
     </row>
-    <row r="38" ht="42" customHeight="1">
+    <row r="38" ht="36" customHeight="1">
       <c r="A38" s="15" t="inlineStr">
         <is>
           <t>HoAlgoSwitch UtranServiceHoSwitch = ON. SERVICEIRHOCFGGROUP InterRatHoState = MUST_HO or PERMIT_HO. Bind QCI on CNOPERATORQCIPARA.</t>
@@ -8393,7 +8527,7 @@
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="28" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Calculation</t>
+          <t xml:space="preserve">  Calculation + example (not a design)</t>
         </is>
       </c>
       <c r="B40" s="29" t="n"/>
@@ -8405,10 +8539,11 @@
       <c r="H40" s="29" t="n"/>
       <c r="I40" s="29" t="n"/>
     </row>
-    <row r="41" ht="42" customHeight="1">
+    <row r="41" ht="48" customHeight="1">
       <c r="A41" s="30" t="inlineStr">
         <is>
-          <t>Target B1. IRAT offload TTT must be &lt; 3 s or the 3 s meas stop kills the report.</t>
+          <t>Target B1. Example: IRAT Mn = −92, Hys = 2, B1_thd = −100.  −94 &gt; −100 → ENTER.
+IRAT offload TTT must be &lt; 3 s or the 3 s meas stop kills the report.</t>
         </is>
       </c>
       <c r="B41" s="29" t="n"/>
@@ -8483,7 +8618,7 @@
       <c r="H48" s="14" t="n"/>
       <c r="I48" s="14" t="n"/>
     </row>
-    <row r="49" ht="42" customHeight="1">
+    <row r="49" ht="36" customHeight="1">
       <c r="A49" s="15" t="inlineStr">
         <is>
           <t>HoAlgoSwitch GeranServiceHoSwitch = ON. Same SERVICEIRHOCFGGROUP bind as 6.3.</t>
@@ -9344,7 +9479,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="28" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Calculation</t>
+          <t xml:space="preserve">  Calculation + example (not a design)</t>
         </is>
       </c>
       <c r="B18" s="29" t="n"/>
@@ -9356,13 +9491,15 @@
       <c r="H18" s="29" t="n"/>
       <c r="I18" s="29" t="n"/>
     </row>
-    <row r="19" ht="98" customHeight="1">
+    <row r="19" ht="112" customHeight="1">
       <c r="A19" s="30" t="inlineStr">
         <is>
           <t>Distance from TA. Precision about 100 to 150 m.
 Start: measured distance &gt; DistBasedHoThd for 10 seconds.
 Stop: measured distance ≤ stop threshold for 10 seconds.
-LTE target A4: InterFreqHoA4ThdRSRP / RSRQ (same A4 as coverage IFHO). Must still be better than coverage A2.</t>
+LTE target A4: InterFreqHoA4ThdRSRP / RSRQ (same A4 as coverage IFHO). Must still be better than coverage A2.
+Example: DistBasedHoThd = 3000 m. TA says 3200 m for 10 s → start. Then A4: Mn = −90 dBm, Hys = 2, A4 = −105 dBm.  −92 &gt; −105 → HO to the planned layer.
+If TA later falls to 2500 m for 10 s → stop distance measurement. Do not wait for coverage A2 on an overshoot lobe.</t>
         </is>
       </c>
       <c r="B19" s="29" t="n"/>
@@ -9399,7 +9536,7 @@
       <c r="H24" s="14" t="n"/>
       <c r="I24" s="14" t="n"/>
     </row>
-    <row r="25" ht="42" customHeight="1">
+    <row r="25" ht="36" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
         <is>
           <t>CELLALGOSWITCH DistBasedHoSwitch = ON. DISTBASEDHO DistBasedMeasObjType EUTRAN = selected.</t>
@@ -9511,7 +9648,7 @@
       <c r="H34" s="14" t="n"/>
       <c r="I34" s="14" t="n"/>
     </row>
-    <row r="35" ht="42" customHeight="1">
+    <row r="35" ht="36" customHeight="1">
       <c r="A35" s="15" t="inlineStr">
         <is>
           <t>DistBasedHoSwitch = ON. DistBasedMeasObjType UTRAN-1 and/or GERAN-1. Target B1.</t>
@@ -9542,7 +9679,7 @@
       <c r="H37" s="32" t="n"/>
       <c r="I37" s="32" t="n"/>
     </row>
-    <row r="38" ht="42" customHeight="1">
+    <row r="38" ht="36" customHeight="1">
       <c r="A38" s="33" t="inlineStr">
         <is>
           <t>Chapter 4 IRAT neighbours. Coverage IRAT is still the edge rescue; this is overshoot only.</t>
@@ -10141,7 +10278,7 @@
       <c r="H20" s="14" t="n"/>
       <c r="I20" s="14" t="n"/>
     </row>
-    <row r="21" ht="42" customHeight="1">
+    <row r="21" ht="36" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
           <t>ENODEBALGOSWITCH HoAlgoSwitch UlQualityInterFreqHoSwitch = ON.</t>
@@ -10160,7 +10297,7 @@
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="28" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Calculation</t>
+          <t xml:space="preserve">  Calculation + example (not a design)</t>
         </is>
       </c>
       <c r="B23" s="29" t="n"/>
@@ -10172,13 +10309,15 @@
       <c r="H23" s="29" t="n"/>
       <c r="I23" s="29" t="n"/>
     </row>
-    <row r="24" ht="110" customHeight="1">
+    <row r="24" ht="128" customHeight="1">
       <c r="A24" s="30" t="inlineStr">
         <is>
           <t>Start meas:  UL MCS index &lt; UlBadQualMcsThd   AND   (actual IBLER − target IBLER) &gt; UlBadQualIblerThd
 Stop meas:  MCS ≥ MCS thd   OR   IBLER gap ≤ IBLER thd
 A4 threshold = InterFreqHoA4ThdRSRP + UlBadQualHoA4Offset   (same for RSRQ + offset)
-Blind: MCS &lt; blind MCS thd  AND  (IBLER gap − 10%) &gt; IBLER thd  AND  no A4 received.
+Example start: MCS thd = 6, IBLER thd = 5%. UE MCS = 4, actual IBLER = 12%, target IBLER = 10%.  4 &lt; 6 AND (12−10)=2% &gt; 5%?  2% &gt; 5% is NO, so measurement does not start yet (IBLER not bad enough).
+If actual IBLER = 18%: gap = 8% &gt; 5% AND MCS 4 &lt; 6 → START. Then A4: base −105 dBm + UlBadQualHoA4Offset −3 dB → used A4 = −108 dBm. Mn −90, Hys 2.  −92 &gt; −108 → HO.
+Blind: MCS &lt; blind MCS thd  AND  (IBLER gap − 10%) &gt; IBLER thd  AND  no A4 received. Example: gap 18%, thd 5%.  (18−10)=8% &gt; 5% AND still no A4 → blind redirect.
 If the QCI-1 blind switch is ON, QCI-1 may be blind-redirected; release cause to MME is always User Inactivity.</t>
         </is>
       </c>
@@ -10288,7 +10427,7 @@
       <c r="H33" s="14" t="n"/>
       <c r="I33" s="14" t="n"/>
     </row>
-    <row r="34" ht="42" customHeight="1">
+    <row r="34" ht="36" customHeight="1">
       <c r="A34" s="15" t="inlineStr">
         <is>
           <t>HoAlgoSwitch UlQualityInterRATHoSwitch = ON. Target B1 to UTRAN or GERAN.</t>
@@ -10319,7 +10458,7 @@
       <c r="H36" s="32" t="n"/>
       <c r="I36" s="32" t="n"/>
     </row>
-    <row r="37" ht="42" customHeight="1">
+    <row r="37" ht="36" customHeight="1">
       <c r="A37" s="33" t="inlineStr">
         <is>
           <t>Chapter 4 IRAT neighbours. Same MCS/IBLER start as 8.2.</t>
@@ -10894,7 +11033,7 @@
       <c r="H15" s="14" t="n"/>
       <c r="I15" s="14" t="n"/>
     </row>
-    <row r="16" ht="110" customHeight="1">
+    <row r="16" ht="80" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
           <t>Enable the CQI-based inter-frequency HO bit on CELLHOPARACFG / CELLALGOSWITCH (confirm the exact bit name in MAE on this eRAN21.1).
@@ -10916,7 +11055,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="28" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Calculation</t>
+          <t xml:space="preserve">  Calculation + example (not a design)</t>
         </is>
       </c>
       <c r="B18" s="29" t="n"/>
@@ -10928,11 +11067,13 @@
       <c r="H18" s="29" t="n"/>
       <c r="I18" s="29" t="n"/>
     </row>
-    <row r="19" ht="84" customHeight="1">
+    <row r="19" ht="96" customHeight="1">
       <c r="A19" s="30" t="inlineStr">
         <is>
           <t>Start: serving CQI stays below the CQI threshold for the configured period.
 Target A4: Mn + Ofn + Ocn − Hys &gt; A4_thd (+ any CQI-specific A4 offset if the version has one).
+Example: CQI thd = 6, UE CQI = 4 for the CQI timer → start. Serving RSRP may still be −85 dBm (coverage A2 not fired).
+Then A4 = −105 dBm, Mn = −90, Hys = 2.  −92 &gt; −105 → HO. Keep A4 better than coverage A2.
 Stop / ping-pong guard: A4_thd must be better than coverage A2 so the UE is not immediately measured out of the new cell.</t>
         </is>
       </c>
@@ -11048,7 +11189,7 @@
       <c r="H26" s="32" t="n"/>
       <c r="I26" s="32" t="n"/>
     </row>
-    <row r="27" ht="42" customHeight="1">
+    <row r="27" ht="36" customHeight="1">
       <c r="A27" s="33" t="inlineStr">
         <is>
           <t>Requires Ch.4. Does not replace Ch.5 coverage. Confirm license / bit in MAE. Do not copy book example A4 dBm into Value.</t>
@@ -11575,7 +11716,7 @@
       <c r="H15" s="14" t="n"/>
       <c r="I15" s="14" t="n"/>
     </row>
-    <row r="16" ht="98" customHeight="1">
+    <row r="16" ht="80" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
           <t>CELLALGOSWITCH HoAllowedSwitch ServiceReqInterFreqHoSwitch = ON.
@@ -11597,7 +11738,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="28" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Calculation</t>
+          <t xml:space="preserve">  Calculation + example (not a design)</t>
         </is>
       </c>
       <c r="B18" s="29" t="n"/>
@@ -11609,12 +11750,13 @@
       <c r="H18" s="29" t="n"/>
       <c r="I18" s="29" t="n"/>
     </row>
-    <row r="19" ht="110" customHeight="1">
+    <row r="19" ht="96" customHeight="1">
       <c r="A19" s="30" t="inlineStr">
         <is>
           <t>A4 thd = SrvReqHoA4ThdRsrp (+ SrvReqHoA4ThdRsrq if used)  — its own A4, not mixed with coverage A2.
-This A4 must still be better than coverage A2 so coverage measurement does not start immediately after arrival.
-Wait for A4: ServiceIfHoCfgGroup.A4RptWaitingTimer.
+Example: SrvReqHoA4ThdRsrp = −102 dBm, coverage A2 = −110 dBm. Used service-request A4 (−102) is higher than A2 (−110).
+Mn = −90, Hys = 2.  −92 &gt; −102 → ENTER. After HO, serving −90: −90 + 2 = −88 &lt; −110? NO, so coverage measurement does not start immediately.
+Wait for A4: ServiceIfHoCfgGroup.A4RptWaitingTimer. Example 3 s. If no A4 in 3 s, stop gap measurement so user-plane is not stalled.
 VoipExProtSwitch: if ON and VoLTE exception, set up QCI-1 if PERMIT_HO in initial context, then start IF meas after access.</t>
         </is>
       </c>
@@ -11715,7 +11857,7 @@
       <c r="H25" s="32" t="n"/>
       <c r="I25" s="32" t="n"/>
     </row>
-    <row r="26" ht="42" customHeight="1">
+    <row r="26" ht="36" customHeight="1">
       <c r="A26" s="33" t="inlineStr">
         <is>
           <t>Highest-priority QCI among configured QCIs. Serving frequency not already the target. Chapter 4 flags.</t>

</xml_diff>